<commit_message>
Kurullar güncellendi (yeni Excel)
Düzenleme Kurulu: +Muhammet Enes YANIK, +Özgür Aydın BEKAR
Bilim Kurulu: -Vedat KARADENİZ, -M.E. YANIK, -Ö.A. BEKAR
kurullar.xlsx güncellendi

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mehme\OneDrive\Desktop\Çalıştay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3FA739B-FC19-43DD-A534-E4095548DF28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F2E820E-11DE-4331-AC8F-5EF62142CAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="640" yWindow="990" windowWidth="32710" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="80">
   <si>
     <t>Uluslararası Katılımlı "Erzincan Jeolojik ve Kültürel Miras" Çalıştayı — Kurullar</t>
   </si>
@@ -833,7 +833,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -862,12 +862,6 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -902,6 +896,60 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -923,70 +971,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1289,7 +1277,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.90625" bestFit="1" customWidth="1"/>
@@ -1297,29 +1285,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25"/>
+      <c r="B2" s="41"/>
     </row>
     <row r="3" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="25"/>
+      <c r="B4" s="41"/>
     </row>
     <row r="5" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="11" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1340,384 +1328,376 @@
       </c>
     </row>
     <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="32" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="11" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="25"/>
+      <c r="B11" s="41"/>
     </row>
     <row r="12" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="13" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="17" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="19" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="17" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="25" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="28" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="25" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="28" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="44" t="s">
+      <c r="B22" s="35" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="36" t="s">
+    <row r="23" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B23" s="28" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="38" t="s">
+    <row r="24" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="B22" s="34" t="s">
+      <c r="B24" s="25" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="33" t="s">
+    <row r="25" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B25" s="17" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="32" t="s">
+    <row r="26" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="35" t="s">
+      <c r="B26" s="26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="22" t="s">
+    <row r="27" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B27" s="21" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="28" t="s">
+    <row r="28" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" spans="1:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="25"/>
-    </row>
-    <row r="28" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="16" t="s">
+      <c r="B29" s="41"/>
+    </row>
+    <row r="30" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B30" s="15" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B40" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="48" t="s">
+    <row r="41" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="36" t="s">
         <v>79</v>
       </c>
-      <c r="B39" s="49" t="s">
+      <c r="B41" s="37" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="50" t="s">
+    <row r="42" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="51" t="s">
+      <c r="B42" s="39" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B41" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="7" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="7" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B53" s="9" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="46" t="s">
+    <row r="54" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="B52" s="47" t="s">
+      <c r="B54" s="48" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="B53" s="45" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B55" s="11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B56" s="1"/>
-    </row>
-    <row r="57" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="26"/>
-      <c r="B57" s="25"/>
+    <row r="55" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="1"/>
+    </row>
+    <row r="56" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="42"/>
+      <c r="B56" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A29:B29"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A11:B11"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fatih ORHAN + Ozan Arif KESİK eklendi, Kazancı isim düzeltmesi
Düzenleme Kurulu:
- Fatih ORHAN: Vedat KARADENİZ altına (EBYÜ, Coğrafya)
- Ozan Arif KESİK: Özgür Aydın BEKAR altına (EBYÜ, Coğrafya)
- 3 dilde (TR/EN/IT) i18n kurul listeleri güncellendi
- speaker-name word-break eklendi (uzun isim taşması düzeltildi)
- kurullar.xlsx güncellendi

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -1070,7 +1070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="41.90625" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
@@ -1266,7 +1266,7 @@
     <row r="20" ht="18" customHeight="1" s="41">
       <c r="A20" s="29" t="inlineStr">
         <is>
-          <t>Muhammet Enes YANIK</t>
+          <t>Fatih ORHAN</t>
         </is>
       </c>
       <c r="B20" s="25" t="inlineStr">
@@ -1278,7 +1278,7 @@
     <row r="21" ht="18" customHeight="1" s="41">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>Özgür Aydın BEKAR</t>
+          <t>Muhammet Enes YANIK</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
@@ -1290,80 +1290,96 @@
     <row r="22" ht="18" customHeight="1" s="41">
       <c r="A22" s="34" t="inlineStr">
         <is>
-          <t>Erdal SARIGÜL</t>
+          <t>Özgür Aydın BEKAR</t>
         </is>
       </c>
       <c r="B22" s="35" t="inlineStr">
         <is>
-          <t>TMMOB Jeoloji Mühendisleri Odası Erzincan Temsilciliği</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan-Türkiye</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="41">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>Murat GÖMÜÇ</t>
+          <t>Ozan Arif KESİK</t>
         </is>
       </c>
       <c r="B23" s="28" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Doktora Öğrencisi</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan-Türkiye</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="41">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>Halil İbrahim DÖNMEZ</t>
+          <t>Erdal SARIGÜL</t>
         </is>
       </c>
       <c r="B24" s="25" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Doktora Öğrencisi</t>
+          <t>TMMOB Jeoloji Mühendisleri Odası Erzincan Temsilciliği</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="41">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>Rukiye ÖZ</t>
+          <t>Murat GÖMÜÇ</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Yüksek Lisans Öğrencisi</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Doktora Öğrencisi</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="41">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>Eren KUTLUDİL</t>
+          <t>Halil İbrahim DÖNMEZ</t>
         </is>
       </c>
       <c r="B26" s="26" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Kulübü Başkanı</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Doktora Öğrencisi</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="41">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>Berkan ÖKSÜZ</t>
+          <t>Rukiye ÖZ</t>
         </is>
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>İstanbul Üniversitesi-Cerrahpaşa, Jeoloji Kulübü</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="6" customHeight="1" s="41"/>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Yüksek Lisans Öğrencisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="6" customHeight="1" s="41">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Eren KUTLUDİL</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Kulübü Başkanı</t>
+        </is>
+      </c>
+    </row>
     <row r="29" ht="25" customHeight="1" s="41">
       <c r="A29" s="44" t="inlineStr">
         <is>
-          <t>🔬 BİLİM KURULU / Scientific Committee</t>
+          <t>Berkan ÖKSÜZ</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>İstanbul Üniversitesi-Cerrahpaşa, Jeoloji Kulübü</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1398,7 @@
     <row r="31" ht="18" customHeight="1" s="41">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Ali DEMİRSOY</t>
+          <t>🔬 BİLİM KURULU / Scientific Committee</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1394,294 +1410,306 @@
     <row r="32" ht="18" customHeight="1" s="41">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Ali ERGEN</t>
+          <t>İSİM</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>MTA Genel Müdürlüğü, Jeoloji Etütleri Dairesi, Ankara</t>
+          <t>KURUM</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" s="41">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Ali KANDEMİR</t>
+          <t>Ali DEMİRSOY</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Biyoloji Bölümü, Erzincan</t>
+          <t>Hacettepe Üniversitesi, Fen Fakültesi, Biyoloji Bölümü, Ankara</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1" s="41">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Enrico CAPEZZUOLİ</t>
+          <t>Ali ERGEN</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Università di Firenze, Dipartimento di Scienze della Terra /Floransa Üniversitesi, Yer Bilimleri Bölümü, İtalya</t>
+          <t>MTA Genel Müdürlüğü, Jeoloji Etütleri Dairesi, Ankara</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="41">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Erdal AKPINAR</t>
+          <t>Ali KANDEMİR</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Biyoloji Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="41">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Eşref ATABEY</t>
+          <t>Enrico CAPEZZUOLİ</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Tıbbi Jeoloji Uzmanı</t>
+          <t>Università di Firenze, Dipartimento di Scienze della Terra /Floransa Üniversitesi, Yer Bilimleri Bölümü, İtalya</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" s="41">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Ezher TAGLİASACCHİ</t>
+          <t>Erdal AKPINAR</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Pamukkale Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Denizli</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" s="41">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Fatma ŞİŞMAN TÜKEL</t>
+          <t>Eşref ATABEY</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, İstanbul</t>
+          <t>Tıbbi Jeoloji Uzmanı</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="41">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Gülpınar AKBULUT</t>
+          <t>Ezher TAGLİASACCHİ</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Sivas Cumhuriyet Üniversitesi, Türkçe ve Sosyal Bilimler Eğitimi Bölümü, Coğrafya Eğitimi ABD</t>
+          <t>Pamukkale Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Denizli</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" s="41">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>İbrahim KOPAR</t>
+          <t>Fatma ŞİŞMAN TÜKEL</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Atatürk Üniversitesi, Edebiyat Fakültesi, Coğrafya Bölümü, Erzurum</t>
+          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, İstanbul</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="41">
       <c r="A41" s="36" t="inlineStr">
         <is>
-          <t>İbrahim ÜNGÖR</t>
+          <t>Gülpınar AKBULUT</t>
         </is>
       </c>
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Tarih Bölümü, Erzincan</t>
+          <t>Sivas Cumhuriyet Üniversitesi, Türkçe ve Sosyal Bilimler Eğitimi Bölümü, Coğrafya Eğitimi ABD</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1" s="41">
       <c r="A42" s="38" t="inlineStr">
         <is>
-          <t>Kenan İNAN</t>
+          <t>İbrahim KOPAR</t>
         </is>
       </c>
       <c r="B42" s="39" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Tarih Bölümü, Erzincan</t>
+          <t>Atatürk Üniversitesi, Edebiyat Fakültesi, Coğrafya Bölümü, Erzurum</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1" s="41">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Kuttusi Zorlu</t>
+          <t>İbrahim ÜNGÖR</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Tarih Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" s="41">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Mehmet Akif TAŞ</t>
+          <t>Kenan İNAN</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Tarih Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1" s="41">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Murat USLU</t>
+          <t>Kuttusi Zorlu</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>Erzurum Vakıflar Bölge Müdürlüğü, Erzurum</t>
+          <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1" s="41">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Mustafa BAYAM</t>
+          <t>Mehmet Akif TAŞ</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Erzincan Müze Müdürlüğü, Erzincan</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1" s="41">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Mustafa Feridun ÇELİKMEN</t>
+          <t>Murat USLU</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>Kemaliye Kültür ve Kalkınma Vakfı (KEMAV) Başkanı, Erzincan</t>
+          <t>Erzurum Vakıflar Bölge Müdürlüğü, Erzurum</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1" s="41">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Nizamettin KAZANCI</t>
+          <t>Mustafa BAYAM</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>JEMİRKO Başkanı, UNESCO Türkiye Milli Komisyonu Başkan Vekili</t>
+          <t>Erzincan Müze Müdürlüğü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1" s="41">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Pınar POLAT</t>
+          <t>Mustafa Feridun ÇELİKMEN</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
+          <t>Kemaliye Kültür ve Kalkınma Vakfı (KEMAV) Başkanı, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="41">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Raif KANDEMİR</t>
+          <t>Nizamettin KAZANCI</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Karadeniz Teknik Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Trabzon</t>
+          <t>JEMİRKO Başkanı, UNESCO Türkiye Milli Komisyonu Başkan Vekili</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1" s="41">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Samet ALTINBİLEK</t>
+          <t>Pınar POLAT</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi,  Sosyal Bilimler ve Türkçe Eğitimi Bölümü, Erzincan</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" s="41">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>Volkan DEDE</t>
+          <t>Raif KANDEMİR</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
+          <t>Karadeniz Teknik Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Trabzon</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" s="41">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Yakup ÇELİK</t>
+          <t>Samet ALTINBİLEK</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi,  Sosyal Bilimler ve Türkçe Eğitimi Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" s="41">
       <c r="A54" s="47" t="inlineStr">
         <is>
+          <t>Volkan DEDE</t>
+        </is>
+      </c>
+      <c r="B54" s="48" t="inlineStr">
+        <is>
+          <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="6" customHeight="1" s="41">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Yakup ÇELİK</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1" s="41">
+      <c r="A56" s="42" t="inlineStr">
+        <is>
           <t>Yıldırım GÜNGÖR</t>
         </is>
       </c>
-      <c r="B54" s="48" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="6" customHeight="1" s="41">
-      <c r="B55" s="1" t="n"/>
-    </row>
-    <row r="56" ht="20" customHeight="1" s="41">
-      <c r="A56" s="42" t="n"/>
-    </row>
+    <row r="57"/>
+    <row r="58"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A56:B56"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>

</xml_diff>

<commit_message>
Detaylı denetim düzeltmeleri (site + 3 xlsx)
Site: stat 21+ -> 18 (gerçek sunum sayısı); FAQ static salon adı Büyükkasap'a (i18n ile aynı); Bilim Kurulu static fallback sırası i18n ile eşitlendi; Vedat Güngör kart rolü 3 dilde yerelleştirildi (sp_role_vgungor); kayıt formuna mode:no-cors; M.A.Taş kartına Polat Gölü bildirisi; IT galeri etiketi Monte Esence; EN/IT gün sekmesi tam ay adı.

xlsx: kurullar orijinalden temiz yeniden kuruldu (önceki insert_rows'un Eren Kutludil satırını bozması + hatalı A31:B31 birleştirmesi giderildi), Bilim Taş/Seven sırası siteyle eşit, Kenan İNAN büyük harf; program EN tablo: Nene Hatun->Mamahatun, Cuma gala (Ergan Zirve), Cmt düz akşam yemeği; sunum row 10 başlık dolduruldu.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -1186,7 +1186,7 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>Kenan İnan (Fen-Edebiyat Fak. Dekanı)</t>
+          <t>Kenan İNAN (Fen-Edebiyat Fak. Dekanı)</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
@@ -1636,24 +1636,24 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="33" t="inlineStr">
         <is>
-          <t>Mutlu SEVEN</t>
+          <t>Mehmet Akif TAŞ</t>
         </is>
       </c>
       <c r="B49" s="34" t="inlineStr">
         <is>
-          <t>Kilis 7 Aralık Üniversitesi, İnsan ve Toplum Bilimleri Fakültesi, Coğrafya Bölümü</t>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="35" t="inlineStr">
         <is>
-          <t>Mehmet Akif TAŞ</t>
+          <t>Mutlu SEVEN</t>
         </is>
       </c>
       <c r="B50" s="36" t="inlineStr">
         <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
+          <t>Kilis 7 Aralık Üniversitesi, İnsan ve Toplum Bilimleri Fakültesi, Coğrafya Bölümü</t>
         </is>
       </c>
     </row>
@@ -1790,12 +1790,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A31:B31"/>
     <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Denetim kararları uygulandı (kullanıcı onayı)
1) Kuddusi -> Kuttusi (oturum+timeline+sunum.xlsx). 4) TAGLİASACCHİ -> TAGLIASACCHI düz yazım (Bilim static+kart+i18n 3 dil; kurullar+sunum.xlsx). 5) Tükel bildirisi tam başlığa ('Kuzey Anadolu Fayı'nın Magmatik İzlerinden Jeolojik Mirasa: ...'). 6) Capezzuoli sunum.xlsx başlığı İngilizce'ye (site ile aynı). Ek: kurullar Kuttusi ZORLU büyük harf, sunum Fatma Şişman TÜKEL + ortak yazarlar. (2 gmail, 3 Vedat'lar: değişiklik yok — doğru.)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -1552,7 +1552,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Ezher TAGLİASACCHİ</t>
+          <t>Ezher TAGLIASACCHI</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
@@ -1624,7 +1624,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Kuttusi Zorlu</t>
+          <t>Kuttusi ZORLU</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Kurul güncellemeleri + TEKDER sponsor + poster yenileme
Düzenleme Kurulu: +Ali Ergen (Erdal Sarıgül altına; site 3 dil + kurullar.xlsx). Bilim Kurulu: +Serdar Akgündüz, İstanbul Üni.-Cerrahpaşa (alfabetik, Samet Altınbilek'ten sonra; site 3 dil + kurullar.xlsx). Sponsorlara TEKDER (Teknik Elemanlar Derneği İstanbul Şubesi) logosu — LOG.pdf'ten alttaki logo çıkarıldı (Logolar/tekder.png) + sp_tekder i18n 3 dil. Posterler TR+EN yeniden yüklendi (2000px) ve cache-bust artırıldı (tr v8->v9, en v6->v7).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -1105,7 +1105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="53.36328125" customWidth="1" min="1" max="1"/>
@@ -1373,45 +1373,45 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Ali ERGEN</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>MTA Genel Müdürlüğü, Jeoloji Etütleri Dairesi, Ankara</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>Murat GÖMÜÇ</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Doktora Öğrencisi</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="27" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>Halil İbrahim DÖNMEZ</t>
         </is>
       </c>
-      <c r="B27" s="28" t="inlineStr">
+      <c r="B28" s="28" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Doktora Öğrencisi</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>Rukiye ÖZ</t>
-        </is>
-      </c>
-      <c r="B28" s="21" t="inlineStr">
-        <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Yüksek Lisans Öğrencisi</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>Melike BEKAR</t>
+          <t>Rukiye ÖZ</t>
         </is>
       </c>
       <c r="B29" s="21" t="inlineStr">
@@ -1423,367 +1423,391 @@
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
+          <t>Melike BEKAR</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Yüksek Lisans Öğrencisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
           <t>Ayşegül KESİK</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Bölümü, Yüksek Lisans Öğrencisi</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="40" t="inlineStr">
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="40" t="inlineStr">
         <is>
           <t>Eren KUTLUDİL</t>
         </is>
       </c>
-      <c r="B31" s="42" t="inlineStr">
+      <c r="B32" s="42" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Coğrafya Kulübü Başkanı</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="41" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="41" t="inlineStr">
         <is>
           <t>Berkan ÖKSÜZ</t>
         </is>
       </c>
-      <c r="B32" s="43" t="inlineStr">
+      <c r="B33" s="43" t="inlineStr">
         <is>
           <t>İstanbul Üniversitesi-Cerrahpaşa, Jeoloji Kulübü</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1"/>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="55" t="inlineStr">
+    <row r="34" ht="18" customHeight="1"/>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="55" t="inlineStr">
         <is>
           <t>🔬 BİLİM KURULU / Scientific Committee</t>
         </is>
       </c>
-      <c r="B34" s="56" t="n"/>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="45" t="inlineStr">
+      <c r="B35" s="56" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="45" t="inlineStr">
         <is>
           <t>İSİM</t>
         </is>
       </c>
-      <c r="B35" s="44" t="inlineStr">
+      <c r="B36" s="44" t="inlineStr">
         <is>
           <t>KURUM</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="35" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="35" t="inlineStr">
         <is>
           <t>Ali DEMİRSOY</t>
         </is>
       </c>
-      <c r="B36" s="36" t="inlineStr">
+      <c r="B37" s="36" t="inlineStr">
         <is>
           <t>Hacettepe Üniversitesi, Fen Fakültesi, Biyoloji Bölümü, Ankara</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Ali ERGEN</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>MTA Genel Müdürlüğü, Jeoloji Etütleri Dairesi, Ankara</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Ali KANDEMİR</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Biyoloji Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Enrico CAPEZZUOLİ</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Università di Firenze, Dipartimento di Scienze della Terra /Floransa Üniversitesi, Yer Bilimleri Bölümü, İtalya</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>Erdal AKPINAR</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Eşref ATABEY</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Tıbbi Jeoloji Uzmanı</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>Ezher TAGLIASACCHI</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>Pamukkale Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Denizli</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Fatma ŞİŞMAN TÜKEL</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, İstanbul</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="29" t="inlineStr">
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="29" t="inlineStr">
         <is>
           <t>Gülpınar AKBULUT</t>
         </is>
       </c>
-      <c r="B44" s="30" t="inlineStr">
+      <c r="B45" s="30" t="inlineStr">
         <is>
           <t>Sivas Cumhuriyet Üniversitesi, Türkçe ve Sosyal Bilimler Eğitimi Bölümü, Coğrafya Eğitimi ABD</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="31" t="inlineStr">
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="31" t="inlineStr">
         <is>
           <t>İbrahim KOPAR</t>
         </is>
       </c>
-      <c r="B45" s="32" t="inlineStr">
+      <c r="B46" s="32" t="inlineStr">
         <is>
           <t>Atatürk Üniversitesi, Edebiyat Fakültesi, Coğrafya Bölümü, Erzurum</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>İbrahim ÜNGÖR</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Tarih Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="6" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Kenan İNAN</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen-Edebiyat Fakültesi, Tarih Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Kuttusi ZORLU</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="33" t="inlineStr">
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="33" t="inlineStr">
         <is>
           <t>Mehmet Akif TAŞ</t>
         </is>
       </c>
-      <c r="B49" s="34" t="inlineStr">
+      <c r="B50" s="34" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="35" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="35" t="inlineStr">
         <is>
           <t>Mutlu SEVEN</t>
         </is>
       </c>
-      <c r="B50" s="36" t="inlineStr">
+      <c r="B51" s="36" t="inlineStr">
         <is>
           <t>Kilis 7 Aralık Üniversitesi, İnsan ve Toplum Bilimleri Fakültesi, Coğrafya Bölümü</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Murat USLU</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>Erzurum Vakıflar Bölge Müdürlüğü, Erzurum</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Mustafa BAYAM</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B53" s="8" t="inlineStr">
         <is>
           <t>Erzincan Müze Müdürlüğü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Mustafa Feridun ÇELİKMEN</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>Kemaliye Kültür ve Kalkınma Vakfı (KEMAV) Başkanı, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Nizamettin KAZANCI</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B55" s="8" t="inlineStr">
         <is>
           <t>JEMİRKO Başkanı, UNESCO Türkiye Milli Komisyonu Başkan Vekili</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Pınar POLAT</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Raif KANDEMİR</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B57" s="8" t="inlineStr">
         <is>
           <t>Karadeniz Teknik Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Trabzon</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>Samet ALTINBİLEK</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi,  Sosyal Bilimler ve Türkçe Eğitimi Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Serdar AKGÜNDÜZ</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>İstanbul Üniversitesi-Cerrahpaşa</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>Volkan DEDE</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>Yahya ÖZTÜRK</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>Van Yüzüncü Yıl Üniversitesi, Sosyal Bilimler Enstitüsü</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="37" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="37" t="inlineStr">
         <is>
           <t>Yakup ÇELİK</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="38" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="38" t="inlineStr">
         <is>
           <t>Yıldırım GÜNGÖR</t>
         </is>
       </c>
-      <c r="B61" s="39" t="inlineStr">
+      <c r="B63" s="39" t="inlineStr">
         <is>
           <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
         </is>
@@ -1795,7 +1819,7 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
Konuşmacı/kurul revizyonu: Dede-Zorlu çıkarıldı, Kazancı en üste, İnan başlığı, kart düzeni
- Volkan Dede + Kuttusi Zorlu her yerden kaldırıldı (kart, Bilim Kurulu
  statik+3 dil, oturum 2 listesi, timeline, kurullar/sunum xlsx);
  Oturum 2 4->3 sunum, toplam 18->17 (site stat + program xlsx TR/EN)
- Erdal Akpınar yalnız davetli kartından çıkarıldı (kurullar/oturum/
  program/xlsx'te duruyor); sp_role_akpinar+sp_role_zorlu 3 dilden silindi
- Nizamettin Kazancı kartı en üste alındı (sunum programındaki ilk isim),
  kalan kartlar alfabetik sıralandı
- Kenan İnan bildiri başlığı eklendi: 'Coğrafya ve Tarih: 1473 Otlukbeli
  Savaşının Yerinin Tespiti ve Yol Güzergahları' (oturum+timeline+kart+xlsx)
- Davetli kartlarına kutu görünümü (arka plan+çerçeve+radius) — boşluklu/
  düzensiz görünüm giderildi

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -1105,7 +1105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="53.36328125" customWidth="1" min="1" max="1"/>
@@ -1634,180 +1634,156 @@
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Kuttusi ZORLU</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
+      <c r="A49" s="33" t="inlineStr">
+        <is>
+          <t>Mehmet Akif TAŞ</t>
+        </is>
+      </c>
+      <c r="B49" s="34" t="inlineStr">
+        <is>
+          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="33" t="inlineStr">
-        <is>
-          <t>Mehmet Akif TAŞ</t>
-        </is>
-      </c>
-      <c r="B50" s="34" t="inlineStr">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Mutlu SEVEN</t>
+        </is>
+      </c>
+      <c r="B50" s="36" t="inlineStr">
+        <is>
+          <t>Kilis 7 Aralık Üniversitesi, İnsan ve Toplum Bilimleri Fakültesi, Coğrafya Bölümü</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Murat USLU</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Erzurum Vakıflar Bölge Müdürlüğü, Erzurum</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Mustafa BAYAM</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Erzincan Müze Müdürlüğü, Erzincan</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Mustafa Feridun ÇELİKMEN</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Kemaliye Kültür ve Kalkınma Vakfı (KEMAV) Başkanı, Erzincan</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Nizamettin KAZANCI</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>JEMİRKO Başkanı, UNESCO Türkiye Milli Komisyonu Başkan Vekili</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Pınar POLAT</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="35" t="inlineStr">
-        <is>
-          <t>Mutlu SEVEN</t>
-        </is>
-      </c>
-      <c r="B51" s="36" t="inlineStr">
-        <is>
-          <t>Kilis 7 Aralık Üniversitesi, İnsan ve Toplum Bilimleri Fakültesi, Coğrafya Bölümü</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>Murat USLU</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Erzurum Vakıflar Bölge Müdürlüğü, Erzurum</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Mustafa BAYAM</t>
-        </is>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>Erzincan Müze Müdürlüğü, Erzincan</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>Mustafa Feridun ÇELİKMEN</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Kemaliye Kültür ve Kalkınma Vakfı (KEMAV) Başkanı, Erzincan</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Nizamettin KAZANCI</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>JEMİRKO Başkanı, UNESCO Türkiye Milli Komisyonu Başkan Vekili</t>
-        </is>
-      </c>
-    </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>Pınar POLAT</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi, Fen Edebiyat Fakültesi, Coğrafya Bölümü, Erzincan</t>
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Raif KANDEMİR</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>Karadeniz Teknik Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Trabzon</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Raif KANDEMİR</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>Karadeniz Teknik Üniversitesi, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü, Trabzon</t>
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Samet ALTINBİLEK</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Erzincan Binali Yıldırım Üniversitesi,  Sosyal Bilimler ve Türkçe Eğitimi Bölümü, Erzincan</t>
         </is>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>Samet ALTINBİLEK</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>Erzincan Binali Yıldırım Üniversitesi,  Sosyal Bilimler ve Türkçe Eğitimi Bölümü, Erzincan</t>
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Serdar AKGÜNDÜZ</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>İstanbul Üniversitesi-Cerrahpaşa</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Serdar AKGÜNDÜZ</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>İstanbul Üniversitesi-Cerrahpaşa</t>
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Yahya ÖZTÜRK</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Van Yüzüncü Yıl Üniversitesi, Sosyal Bilimler Enstitüsü</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>Volkan DEDE</t>
+      <c r="A60" s="37" t="inlineStr">
+        <is>
+          <t>Yakup ÇELİK</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Ardahan Üniversitesi, İnsani Bilimler ve Edebiyat Fakültesi, Coğrafya Bölümü</t>
+          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>Yahya ÖZTÜRK</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>Van Yüzüncü Yıl Üniversitesi, Sosyal Bilimler Enstitüsü</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="37" t="inlineStr">
-        <is>
-          <t>Yakup ÇELİK</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="38" t="inlineStr">
+      <c r="A61" s="38" t="inlineStr">
         <is>
           <t>Yıldırım GÜNGÖR</t>
         </is>
       </c>
-      <c r="B63" s="39" t="inlineStr">
+      <c r="B61" s="39" t="inlineStr">
         <is>
           <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
         </is>

</xml_diff>

<commit_message>
Yemek düzeni, Ergan Mado, posta kodu, kurul düzeltmeleri
- Gala yemeği 1. güne alındı (Esentepe); 2. gün akşam yemeği Ergan Mado
  (Zirve değil); 3. gün değişmedi — site timeline 3 dil + program xlsx TR/EN
- Posta kodu 24100 -> 24002 (kullanıcı teyidi; venue_addr_val 3 dil + statik)
- Düzenleme Kurulu: Ali Ergen, Erdal Sarıgül'ün önüne alındı (statik+3 dil
  + kurullar.xlsx)
- Serdar Akgündüz kurumu Yakup Çelik'inkiyle eşitlendi: 'İstanbul
  Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği
  Bölümü' (4 site bağlamı + kurullar.xlsx)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/kurullar.xlsx
+++ b/fotolar/kurullar.xlsx
@@ -1363,24 +1363,24 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="22" t="inlineStr">
         <is>
-          <t>Erdal SARIGÜL</t>
+          <t>Ali ERGEN</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>TMMOB Jeoloji Mühendisleri Odası Erzincan Temsilciliği</t>
+          <t>MTA Genel Müdürlüğü, Jeoloji Etütleri Dairesi, Ankara</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>Ali ERGEN</t>
+          <t>Erdal SARIGÜL</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>MTA Genel Müdürlüğü, Jeoloji Etütleri Dairesi, Ankara</t>
+          <t>TMMOB Jeoloji Mühendisleri Odası Erzincan Temsilciliği</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>İstanbul Üniversitesi-Cerrahpaşa</t>
+          <t>İstanbul Üniversitesi-Cerrahpaşa, Mühendislik Fakültesi, Jeoloji Mühendisliği Bölümü</t>
         </is>
       </c>
     </row>

</xml_diff>